<commit_message>
Add workbook validation and Orchestrator queue dispatch
</commit_message>
<xml_diff>
--- a/Data/Input/BankStatement_20260917.xlsx
+++ b/Data/Input/BankStatement_20260917.xlsx
@@ -5,15 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://standardbank-my.sharepoint.com/personal/ishaku_danladi_stanbicibtc_com/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ishaku\Documents\UiPath\uipath-bank-reconciliation\Data\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{B8DF62D0-02D8-423E-9B6D-00114D9A8F6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5CAC5EF9-4BA4-4B57-B5F7-04C0FB5FB05A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B003577F-DA7D-4C7D-A9B0-8423B0519B6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Bank Transactions" sheetId="1" r:id="rId1"/>
+    <sheet name="Transactions" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -536,7 +536,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -548,7 +548,7 @@
     <col min="9" max="9" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -577,7 +577,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -606,7 +606,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>14</v>
       </c>
@@ -635,7 +635,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
@@ -664,7 +664,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -693,7 +693,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -722,7 +722,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>26</v>
       </c>
@@ -751,7 +751,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>29</v>
       </c>
@@ -780,7 +780,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>32</v>
       </c>

</xml_diff>